<commit_message>
Cap nhat lai data moi
</commit_message>
<xml_diff>
--- a/01 Datamix.xlsx
+++ b/01 Datamix.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="I:\01 Master\02 Smart Concrete\01 Developing app for predict compressive and tensile strength\ConstructionMaterialsLab\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A154CE1F-24E2-4C28-85FC-8DC4789222F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21833F41-A48F-4FE0-8016-A6CF76223B64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-90" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="27">
   <si>
     <t>Materials</t>
   </si>
@@ -117,6 +117,9 @@
   </si>
   <si>
     <t>Cement</t>
+  </si>
+  <si>
+    <t>WG (Water glass)</t>
   </si>
 </sst>
 </file>
@@ -451,24 +454,24 @@
     <col min="2" max="3" width="19" style="1" customWidth="1"/>
     <col min="4" max="4" width="15.375" style="1" customWidth="1"/>
     <col min="5" max="5" width="12.75" style="1" customWidth="1"/>
-    <col min="6" max="6" width="21.125" style="1" customWidth="1"/>
-    <col min="7" max="8" width="20.125" style="1" customWidth="1"/>
-    <col min="9" max="9" width="15.875" style="1" customWidth="1"/>
-    <col min="10" max="10" width="14.375" style="1" customWidth="1"/>
-    <col min="11" max="11" width="20.25" style="1" customWidth="1"/>
-    <col min="12" max="12" width="17.125" style="1" customWidth="1"/>
-    <col min="13" max="14" width="16.125" style="1" customWidth="1"/>
-    <col min="15" max="15" width="18.375" style="1" customWidth="1"/>
-    <col min="16" max="17" width="15.75" style="1" customWidth="1"/>
-    <col min="18" max="18" width="20" style="1" customWidth="1"/>
-    <col min="19" max="19" width="21.25" style="1" customWidth="1"/>
-    <col min="20" max="20" width="17.375" style="1" customWidth="1"/>
-    <col min="21" max="21" width="18.5" style="1" customWidth="1"/>
-    <col min="22" max="22" width="11.625" style="1" hidden="1" customWidth="1"/>
-    <col min="23" max="16384" width="9" style="1"/>
+    <col min="6" max="7" width="21.125" style="1" customWidth="1"/>
+    <col min="8" max="9" width="20.125" style="1" customWidth="1"/>
+    <col min="10" max="10" width="15.875" style="1" customWidth="1"/>
+    <col min="11" max="11" width="14.375" style="1" customWidth="1"/>
+    <col min="12" max="12" width="20.25" style="1" customWidth="1"/>
+    <col min="13" max="13" width="17.125" style="1" customWidth="1"/>
+    <col min="14" max="15" width="16.125" style="1" customWidth="1"/>
+    <col min="16" max="16" width="18.375" style="1" customWidth="1"/>
+    <col min="17" max="18" width="15.75" style="1" customWidth="1"/>
+    <col min="19" max="19" width="20" style="1" customWidth="1"/>
+    <col min="20" max="20" width="21.25" style="1" customWidth="1"/>
+    <col min="21" max="21" width="17.375" style="1" customWidth="1"/>
+    <col min="22" max="22" width="18.5" style="1" customWidth="1"/>
+    <col min="23" max="23" width="11.625" style="1" hidden="1" customWidth="1"/>
+    <col min="24" max="16384" width="9" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" s="2" customFormat="1" ht="57">
+    <row r="1" spans="1:23" s="2" customFormat="1" ht="57">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -488,55 +491,58 @@
         <v>22</v>
       </c>
       <c r="G1" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="H1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="I1" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="I1" s="3" t="s">
+      <c r="J1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="J1" s="3" t="s">
+      <c r="K1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="K1" s="3" t="s">
+      <c r="L1" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="L1" s="3" t="s">
+      <c r="M1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="M1" s="3" t="s">
+      <c r="N1" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="N1" s="3" t="s">
+      <c r="O1" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="O1" s="3" t="s">
+      <c r="P1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="P1" s="3" t="s">
+      <c r="Q1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="Q1" s="3" t="s">
+      <c r="R1" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="R1" s="3" t="s">
+      <c r="S1" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="S1" s="3" t="s">
+      <c r="T1" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="T1" s="3" t="s">
+      <c r="U1" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="U1" s="3" t="s">
+      <c r="V1" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="V1" s="2" t="s">
+      <c r="W1" s="2" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="2" spans="1:22" s="2" customFormat="1">
+    <row r="2" spans="1:23" s="2" customFormat="1">
       <c r="A2" s="2" t="s">
         <v>17</v>
       </c>
@@ -556,52 +562,55 @@
         <v>2200</v>
       </c>
       <c r="G2" s="2">
+        <v>1370</v>
+      </c>
+      <c r="H2" s="2">
         <v>2620</v>
       </c>
-      <c r="H2" s="2">
+      <c r="I2" s="2">
         <v>2130</v>
       </c>
-      <c r="I2" s="2">
+      <c r="J2" s="2">
         <v>2240</v>
       </c>
-      <c r="J2" s="2">
+      <c r="K2" s="2">
         <v>2660</v>
       </c>
-      <c r="K2" s="2">
+      <c r="L2" s="2">
         <v>2100</v>
       </c>
-      <c r="L2" s="2">
+      <c r="M2" s="2">
         <v>2690</v>
       </c>
-      <c r="M2" s="2">
+      <c r="N2" s="2">
         <v>2600</v>
       </c>
-      <c r="N2" s="2">
+      <c r="O2" s="2">
         <v>1130</v>
       </c>
-      <c r="O2" s="2">
+      <c r="P2" s="2">
         <v>1000</v>
       </c>
-      <c r="P2" s="2">
+      <c r="Q2" s="2">
         <v>1200</v>
       </c>
-      <c r="Q2" s="2">
+      <c r="R2" s="2">
         <v>1000</v>
       </c>
-      <c r="R2" s="2">
+      <c r="S2" s="2">
         <v>1200</v>
       </c>
-      <c r="S2" s="2">
+      <c r="T2" s="2">
         <v>970</v>
       </c>
-      <c r="T2" s="2">
+      <c r="U2" s="2">
         <v>1300</v>
       </c>
-      <c r="U2" s="2">
+      <c r="V2" s="2">
         <v>7800</v>
       </c>
     </row>
-    <row r="3" spans="1:22" s="2" customFormat="1">
+    <row r="3" spans="1:23" s="2" customFormat="1">
       <c r="A3" s="2" t="s">
         <v>11</v>
       </c>
@@ -621,55 +630,58 @@
         <v>3.5999999999999997E-2</v>
       </c>
       <c r="G3" s="2">
+        <v>6</v>
+      </c>
+      <c r="H3" s="2">
         <v>0.33</v>
       </c>
-      <c r="H3" s="2">
+      <c r="I3" s="2">
         <v>18</v>
       </c>
-      <c r="I3" s="2">
+      <c r="J3" s="2">
         <v>4.25</v>
       </c>
-      <c r="J3" s="2">
+      <c r="K3" s="2">
         <v>6</v>
       </c>
-      <c r="K3" s="2">
+      <c r="L3" s="2">
         <v>4.5999999999999996</v>
       </c>
-      <c r="L3" s="2">
+      <c r="M3" s="2">
         <v>7.9600000000000004E-2</v>
       </c>
-      <c r="M3" s="2">
+      <c r="N3" s="2">
         <v>6.7000000000000004E-2</v>
       </c>
-      <c r="N3" s="2">
+      <c r="O3" s="2">
         <v>7</v>
       </c>
-      <c r="O3" s="4">
+      <c r="P3" s="4">
         <v>0</v>
-      </c>
-      <c r="P3" s="2">
-        <v>35</v>
       </c>
       <c r="Q3" s="2">
         <v>35</v>
       </c>
       <c r="R3" s="2">
+        <v>35</v>
+      </c>
+      <c r="S3" s="2">
         <v>4.9800000000000004</v>
       </c>
-      <c r="S3" s="2">
+      <c r="T3" s="2">
         <v>94.5</v>
       </c>
-      <c r="T3" s="2">
+      <c r="U3" s="2">
         <v>101</v>
       </c>
-      <c r="U3" s="2">
+      <c r="V3" s="2">
         <v>60</v>
       </c>
-      <c r="V3" s="2">
+      <c r="W3" s="2">
         <v>6.5</v>
       </c>
     </row>
-    <row r="4" spans="1:22" s="2" customFormat="1">
+    <row r="4" spans="1:23" s="2" customFormat="1">
       <c r="A4" s="2" t="s">
         <v>12</v>
       </c>
@@ -689,55 +701,58 @@
         <v>1.4E-2</v>
       </c>
       <c r="G4" s="2">
+        <v>1.51</v>
+      </c>
+      <c r="H4" s="2">
         <v>0.33200000000000002</v>
       </c>
-      <c r="H4" s="2">
+      <c r="I4" s="2">
         <v>0.86</v>
       </c>
-      <c r="I4" s="2">
+      <c r="J4" s="2">
         <v>1.0900000000000001</v>
       </c>
-      <c r="J4" s="2">
+      <c r="K4" s="2">
         <v>0.47</v>
       </c>
-      <c r="K4" s="2">
+      <c r="L4" s="2">
         <v>0.43</v>
       </c>
-      <c r="L4" s="2">
+      <c r="M4" s="2">
         <v>2.8E-3</v>
       </c>
-      <c r="M4" s="2">
+      <c r="N4" s="2">
         <v>2.3E-2</v>
       </c>
-      <c r="N4" s="2">
+      <c r="O4" s="2">
         <v>2.7</v>
       </c>
-      <c r="O4" s="4">
+      <c r="P4" s="4">
         <v>0</v>
-      </c>
-      <c r="P4" s="2">
-        <v>1.667</v>
       </c>
       <c r="Q4" s="2">
         <v>1.667</v>
       </c>
       <c r="R4" s="2">
+        <v>1.667</v>
+      </c>
+      <c r="S4" s="2">
         <v>0.48</v>
       </c>
-      <c r="S4" s="2">
+      <c r="T4" s="2">
         <v>4.08</v>
       </c>
-      <c r="T4" s="2">
+      <c r="U4" s="2">
         <v>3.4</v>
       </c>
-      <c r="U4" s="2">
+      <c r="V4" s="2">
         <v>1.6</v>
       </c>
-      <c r="V4" s="2">
+      <c r="W4" s="2">
         <v>0.45</v>
       </c>
     </row>
-    <row r="5" spans="1:22" s="2" customFormat="1">
+    <row r="5" spans="1:23" s="2" customFormat="1">
       <c r="A5" s="2" t="s">
         <v>13</v>
       </c>
@@ -757,51 +772,54 @@
         <v>0.3</v>
       </c>
       <c r="G5" s="2">
+        <v>0.53</v>
+      </c>
+      <c r="H5" s="2">
         <v>0.22900000000000001</v>
       </c>
-      <c r="H5" s="2">
+      <c r="I5" s="2">
         <v>0.25</v>
       </c>
-      <c r="I5" s="2">
+      <c r="J5" s="2">
         <v>0.2</v>
       </c>
-      <c r="J5" s="2">
+      <c r="K5" s="2">
         <v>0.25</v>
       </c>
-      <c r="K5" s="2">
+      <c r="L5" s="2">
         <v>0.17</v>
       </c>
-      <c r="L5" s="2">
+      <c r="M5" s="2">
         <v>0.25</v>
       </c>
-      <c r="M5" s="2">
+      <c r="N5" s="2">
         <v>6.3899999999999998E-2</v>
       </c>
-      <c r="N5" s="2">
+      <c r="O5" s="2">
         <v>0.48</v>
       </c>
-      <c r="O5" s="2">
+      <c r="P5" s="2">
         <v>1.5E-3</v>
-      </c>
-      <c r="P5" s="2">
-        <v>1.2110000000000001</v>
       </c>
       <c r="Q5" s="2">
         <v>1.2110000000000001</v>
       </c>
       <c r="R5" s="2">
+        <v>1.2110000000000001</v>
+      </c>
+      <c r="S5" s="2">
         <v>2.5</v>
       </c>
-      <c r="S5" s="2">
+      <c r="T5" s="2">
         <v>22.39</v>
       </c>
-      <c r="T5" s="2">
+      <c r="U5" s="2">
         <v>12.67</v>
       </c>
-      <c r="U5" s="2">
+      <c r="V5" s="2">
         <v>5</v>
       </c>
-      <c r="V5" s="2">
+      <c r="W5" s="2">
         <v>1.5</v>
       </c>
     </row>

</xml_diff>